<commit_message>
Update dashboard: new menu order, per-month history files, collapsible options, Help page; scrub provider names
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TWYDySAGURhagPjRB9vvPw
</commit_message>
<xml_diff>
--- a/sample-data/ข้อมูลสมมติ_IC Benchmark_2026-07.xlsx
+++ b/sample-data/ข้อมูลสมมติ_IC Benchmark_2026-07.xlsx
@@ -944,7 +944,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Morningstar Thailand Index</t>
+          <t>Thailand Index</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -974,7 +974,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Morningstar Thailand Index</t>
+          <t>Thailand Index</t>
         </is>
       </c>
       <c r="D26" t="n">

</xml_diff>